<commit_message>
Show Pearson r with all decimals in annexes 6, 7 and 20
Store the Pearson r values of the Pearson_resumen and Pearson_<rank>
sheets as text with full precision, so spreadsheets do not round them
for display: 0.9915738489565016 (family), 0.9849468218384722 (genus)
and 0.9630498230621352 (species). The values themselves are unchanged.
</commit_message>
<xml_diff>
--- a/Anexo_20_Diferencias_por_familia/Anexo_20_Diferencias_por_familia.xlsx
+++ b/Anexo_20_Diferencias_por_familia/Anexo_20_Diferencias_por_familia.xlsx
@@ -50,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2966,8 +2967,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2987,8 +2991,10 @@
           <t>pearson_r</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>0.9915738489565016</v>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>0.9915738489565016</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -3024,6 +3030,11 @@
   </sheetPr>
   <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3053,14 +3064,20 @@
           <t>Pearson</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>0.9915738489565016</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.9849468218384722</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.9630498230621352</v>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>0.9915738489565016</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>0.9849468218384722</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>0.9630498230621352</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>